<commit_message>
Sanitize sensitive data before release
- Replace example CSVs (balance sheet / income / off-sheet) with fully
  fictitious demo data (虚构'示例制造有限公司'，勾稽平衡) — the previous
  examples were extracted from the company template and contained real amounts
- Regenerate examples/output with the fictitious data
- Remove template cached amounts from the multi-validation report (company
  confidential); keep only the zero-error conclusion
- Verified: no template amounts / company names remain in any tracked file
</commit_message>
<xml_diff>
--- a/examples/output/现金流量表.xlsx
+++ b/examples/output/现金流量表.xlsx
@@ -557,7 +557,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>21,449,673.61</t>
+          <t>2,612,000.00</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr"/>
@@ -589,7 +589,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>157,210.00</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr"/>
@@ -605,7 +605,7 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>21,449,673.61</t>
+          <t>2,769,210.00</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr"/>
@@ -621,7 +621,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>8,055,983.63</t>
+          <t>1,678,400.00</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr"/>
@@ -637,7 +637,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>198,093.27</t>
+          <t>446,810.00</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr"/>
@@ -653,7 +653,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>835,728.00</t>
+          <t>184,000.00</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>12,270,189.52</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr"/>
@@ -685,7 +685,7 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>21,359,994.42</t>
+          <t>2,309,210.00</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr"/>
@@ -701,7 +701,7 @@
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>89,679.19</t>
+          <t>460,000.00</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr"/>
@@ -809,7 +809,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>290,000.00</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr"/>
@@ -857,7 +857,7 @@
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>290,000.00</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr"/>
@@ -873,7 +873,7 @@
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>-290,000.00</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr"/>
@@ -965,7 +965,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>50,000.00</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr"/>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>50,000.00</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr"/>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>-50,000.00</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr"/>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>89,679.19</t>
+          <t>120,000.00</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr"/>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>5,646,774.15</t>
+          <t>255,000.00</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr"/>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>5,000.00</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr"/>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>120,000.00</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr"/>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>20,000.00</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr"/>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t>5,000.00</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr"/>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>80,000.00</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr"/>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>-12,628,409.87</t>
+          <t>-120,000.00</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr"/>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>7,071,314.91</t>
+          <t>125,000.00</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr"/>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>-100.00</t>
+          <t>-30,000.00</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr"/>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>89,679.19</t>
+          <t>460,000.00</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr"/>
@@ -1428,28 +1428,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>✓ 资产负债表勾稽（资产=负债+权益）：年初：资产(67,132,409.28) vs 负债权益(67,132,409.28) ✓；期末：资产(79,850,498.34) vs 负债权益(79,850,498.34) ✓</t>
+          <t>✓ 资产负债表勾稽（资产=负债+权益）：年初：资产(3,150,000.00) vs 负债权益(3,150,000.00) ✓；期末：资产(3,480,000.00) vs 负债权益(3,480,000.00) ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>✓ 经营活动现金流量净额（主表=补充资料）：主表(89,679.19) vs 补充资料(89,679.19)</t>
+          <t>✓ 经营活动现金流量净额（主表=补充资料）：主表(460,000.00) vs 补充资料(460,000.00)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>✓ 现金及现金等价物净增加额（=货币资金及现金等价物变动）：主表(89,679.19) vs 货币资金变动(89,679.19)</t>
+          <t>✓ 现金及现金等价物净增加额（=货币资金及现金等价物变动）：主表(120,000.00) vs 货币资金变动(120,000.00)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>✓ 未分配利润变动 vs 净利润（提示）：未分配利润增加(5,646,774.15) vs 本年净利润(5,646,774.15)；差异通常为利润分配，属正常</t>
+          <t>✓ 未分配利润变动 vs 净利润（提示）：未分配利润增加(255,000.00) vs 本年净利润(255,000.00)；差异通常为利润分配，属正常</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>- “收到的其他与经营活动有关的现金”（平衡项）为负(-12,270,189.52)，已按正数(12,270,189.52)转入“支付的其他与经营活动有关的现金”</t>
+          <t>- “借款所收到的现金”为负(-50,000.00)，已转入“偿还债务所支付的现金”</t>
         </is>
       </c>
     </row>
@@ -1477,35 +1477,35 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>- 支付的各项税费 = 应交增值税(835,728.00) + 其他各项税(0.00) + 所得税(0.00) + 管理税金(0.00) + 其他业务税金(0.00) - 应交税费及应交款增加(0.00)</t>
+          <t>- 支付的各项税费 = 应交增值税(104,000.00) + 其他各项税(20,000.00) + 所得税(55,000.00) + 管理税金(0.00) + 其他业务税金(0.00) - 应交税费及应交款增加(-5,000.00)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>- 销售商品、提供劳务收到的现金 = 营业收入(13,928,800.00)×(1+13%) + (应收票据年初-0.00期末:0.00) + (应收账款年初-期末:-2,968,354.39) + (预收款项期末-年初:8,678,484.00) - 贴现利息(0.00)</t>
+          <t>- 销售商品、提供劳务收到的现金 = 营业收入(2,400,000.00)×(1+13%) + (应收票据年初-150,000.00期末:120,000.00) + (应收账款年初-期末:-150,000.00) + (预收款项期末-年初:20,000.00) - 贴现利息(0.00)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>- 购买商品、接受劳务支付的现金 = (营业成本(7,916,788.35)+存货增加(0.00))×(1+17%) + (应付票据年初-期末:0.00) + (应付账款年初-期末:-1,206,658.74) + (预付款项期末-年初:0.00)</t>
+          <t>- 购买商品、接受劳务支付的现金 = (营业成本(1,600,000.00)+存货增加(-80,000.00))×(1+17%) + (应付票据年初-期末:20,000.00) + (应付账款年初-期末:-120,000.00) + (预付款项期末-年初:0.00)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>- 购建固定资产、无形资产和其他长期资产所支付的现金 = 固定资产增加(0.00) + 工程物资增加(0.00) + 在建工程增加(0.00) + 无形资产及长期资产增加(0.00)</t>
+          <t>- 购建固定资产、无形资产和其他长期资产所支付的现金 = 固定资产增加(300,000.00) + 工程物资增加(0.00) + 在建工程增加(0.00) + 无形资产及长期资产增加(-10,000.00)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>- 收到的其他与经营活动有关的现金（平衡项）= 现金及现金等价物净增加额(89,679.19) + 经营流出小计(9,089,804.90) - 销售商品收到现金(21,449,673.61) - 收到税费返还(0.00) - 投资活动净额(0.00) - 筹资活动净额(0.00) - 汇率影响(0.00)</t>
+          <t>- 收到的其他与经营活动有关的现金（平衡项）= 现金及现金等价物净增加额(120,000.00) + 经营流出小计(2,309,210.00) - 销售商品收到现金(2,612,000.00) - 收到税费返还(0.00) - 投资活动净额(-290,000.00) - 筹资活动净额(-50,000.00) - 汇率影响(0.00)</t>
         </is>
       </c>
     </row>

</xml_diff>